<commit_message>
fix: fix master kanban import
</commit_message>
<xml_diff>
--- a/template_file/MasterExportTemplate.xlsx
+++ b/template_file/MasterExportTemplate.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28827"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98940214-E9E6-42C4-864D-4C2B67150D36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E104F627-CAE9-4EDD-87B9-51954114CBAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-4905" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -238,7 +238,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -254,22 +254,17 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -633,7 +628,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" customWidth="1"/>
@@ -655,23 +650,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="11"/>
     </row>
     <row r="2" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
@@ -698,7 +693,7 @@
       <c r="E4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="7" t="s">
         <v>6</v>
       </c>
       <c r="G4" s="4" t="s">
@@ -733,148 +728,130 @@
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="11"/>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
+      <c r="A5" s="9"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
       <c r="D5" s="12"/>
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
-      <c r="G5" s="11"/>
+      <c r="G5" s="13"/>
       <c r="H5" s="12"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="13"/>
-      <c r="L5" s="14"/>
-      <c r="M5" s="14"/>
-      <c r="N5" s="14"/>
-      <c r="O5" s="14"/>
-      <c r="P5" s="14"/>
+      <c r="I5" s="13"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="12"/>
+      <c r="L5" s="13"/>
+      <c r="M5" s="13"/>
+      <c r="N5" s="13"/>
+      <c r="O5" s="13"/>
+      <c r="P5" s="13"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" s="10"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="10"/>
-      <c r="M6" s="10"/>
-      <c r="N6" s="10"/>
-      <c r="O6" s="10"/>
-      <c r="P6" s="10"/>
+      <c r="A6" s="8"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="8"/>
+      <c r="P6" s="8"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="10"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="10"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="10"/>
-      <c r="O7" s="10"/>
-      <c r="P7" s="10"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="10"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
-      <c r="O8" s="10"/>
-      <c r="P8" s="10"/>
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="10"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10"/>
-      <c r="O9" s="10"/>
-      <c r="P9" s="10"/>
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="10"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="10"/>
-      <c r="N10" s="10"/>
-      <c r="O10" s="10"/>
-      <c r="P10" s="10"/>
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="10"/>
-      <c r="M11" s="10"/>
-      <c r="N11" s="10"/>
-      <c r="O11" s="10"/>
-      <c r="P11" s="10"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="9"/>
-      <c r="N12" s="9"/>
-      <c r="O12" s="9"/>
-      <c r="P12" s="9"/>
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>